<commit_message>
Complete BAU and Fast Track 2040 transit scenarios
</commit_message>
<xml_diff>
--- a/original-input-data/mvv_gtfs_2037/Infrastructure_measures.xlsx
+++ b/original-input-data/mvv_gtfs_2037/Infrastructure_measures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DavidBerling\Masterarbeit Lokal\WP2\Matsim-example-project-TU-Kurs\original-input-data\mvv_gtfs_2037\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8C73816-95A4-4AC3-B445-83A7E97B397C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85952E1-3C3F-4B1C-832D-3032A38B1162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6983" yWindow="-16297" windowWidth="28995" windowHeight="15675" xr2:uid="{C9EB77A7-838A-4CDA-9FC2-6F0F3DBDABA8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="184">
   <si>
     <t>Definition BAU and FT:
 - Im BAU 2040 werden nur Maßnahmen berücksichtigt, deren Umsetzung bis 2040 bereits unabhängig von einer Olympiabewerbung hinreichend gesichert oder sehr plausibel ist.
@@ -573,6 +573,69 @@
   </si>
   <si>
     <t>Implementation follows the two-line operating concept of the U11 feasibility study. Both lines are generated as separate bidirectional GTFS routes</t>
+  </si>
+  <si>
+    <t>https://www.bahnausbau-muenchen.de/projekt.html?PID=108</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>https://www.bahnausbau-muenchen.de/projekt.html?PID=42</t>
+  </si>
+  <si>
+    <t>https://www.bahnausbau-muenchen.de/regionalzughalt-poccistrasse.html</t>
+  </si>
+  <si>
+    <t>https://www.bahnausbau-muenchen.de/projekt.html?PID=5</t>
+  </si>
+  <si>
+    <t>Laim - Berduxstraße - Obermenzing</t>
+  </si>
+  <si>
+    <t>E 28.a BY; E 28.b BY; N 28.a BY; N 28.b BY; E 56 BY; N 56 BY</t>
+  </si>
+  <si>
+    <t>München Hbf – Poccistraße – München Ost; München Ost – Poccistraße – München Hbf</t>
+  </si>
+  <si>
+    <t>Existing GTFS 2037 timetable and frequencies are retained; Poccistraße is added to matching trips that traverse the München Hbf–München Ost corridor</t>
+  </si>
+  <si>
+    <t>Trips of the listed routes that do not traverse the München Hbf–München Ost corridor remain unchanged</t>
+  </si>
+  <si>
+    <t>Model assumption: all GTFS 2037 regional-train trips assigned to the Rosenheim or Mühldorf corridors and actually running between München Hbf and München Ost receive the new stop. Dwell time and additional running time are derived from comparable regional stops</t>
+  </si>
+  <si>
+    <t>S20; western S-Bahn services during disruptions</t>
+  </si>
+  <si>
+    <t>Existing regular routes retained; diversion and turning movements via Heimeranplatz are not simulated</t>
+  </si>
+  <si>
+    <t>No regular-service frequency change; existing GTFS 2037 timetable retained</t>
+  </si>
+  <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>No published change to the regular-day service pattern was identified. The measure primarily improves operational resilience during disruptions. Because the simulation represents a normal operating day without disruptions, no separate GTFS modification is implemented</t>
+  </si>
+  <si>
+    <t>Existing GTFS 2037 timetable retained; the stop is added to regular S2 trips. No additional departures are generated</t>
+  </si>
+  <si>
+    <t>Express S-Bahn services from Altomünster and Petershausen do not serve Berduxstraße</t>
+  </si>
+  <si>
+    <t>https://www.stmb.bayern.de/assets/stmi/vum/schiene/220519_machbarkeitsstudie_bericht_u06_final.pdf</t>
+  </si>
+  <si>
+    <t>Dwell time and additional running time are derived from comparable S-Bahn stops. The builder must distinguish regular S2 trips from express services</t>
+  </si>
+  <si>
+    <t>S20</t>
   </si>
 </sst>
 </file>
@@ -736,11 +799,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{61883FC4-1D17-4081-8945-EF8683794370}" name="Tabelle4" displayName="Tabelle4" ref="A4:P31" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A4:P31" xr:uid="{61883FC4-1D17-4081-8945-EF8683794370}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="nein"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="6">
       <filters>
         <filter val="ja"/>
@@ -1367,7 +1425,7 @@
       </c>
       <c r="L12" s="7"/>
     </row>
-    <row r="13" spans="1:18" hidden="1">
+    <row r="13" spans="1:18">
       <c r="B13" t="s">
         <v>88</v>
       </c>
@@ -1396,7 +1454,25 @@
         <v>89</v>
       </c>
       <c r="L13" t="s">
-        <v>134</v>
+        <v>165</v>
+      </c>
+      <c r="M13" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="O13" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="P13" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>166</v>
+      </c>
+      <c r="R13" s="10" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -1529,7 +1605,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="17" spans="2:18" hidden="1">
+    <row r="17" spans="2:18">
       <c r="B17" t="s">
         <v>81</v>
       </c>
@@ -1561,13 +1637,16 @@
         <v>134</v>
       </c>
     </row>
-    <row r="18" spans="2:18" hidden="1">
+    <row r="18" spans="2:18">
       <c r="B18" t="s">
         <v>83</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
       </c>
+      <c r="D18" s="10" t="s">
+        <v>183</v>
+      </c>
       <c r="E18" t="s">
         <v>74</v>
       </c>
@@ -1590,16 +1669,37 @@
         <v>84</v>
       </c>
       <c r="L18" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="19" spans="2:18" hidden="1">
+        <v>167</v>
+      </c>
+      <c r="M18" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="N18" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="O18" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="P18" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>167</v>
+      </c>
+      <c r="R18" s="10" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="2:18">
       <c r="B19" t="s">
         <v>86</v>
       </c>
       <c r="C19" t="s">
         <v>56</v>
       </c>
+      <c r="D19" s="10" t="s">
+        <v>164</v>
+      </c>
       <c r="E19" t="s">
         <v>26</v>
       </c>
@@ -1619,7 +1719,25 @@
         <v>114</v>
       </c>
       <c r="L19" t="s">
-        <v>134</v>
+        <v>163</v>
+      </c>
+      <c r="M19" t="s">
+        <v>164</v>
+      </c>
+      <c r="N19" t="s">
+        <v>168</v>
+      </c>
+      <c r="O19" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="P19" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q19" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="R19" s="13" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="20" spans="2:18">
@@ -1690,7 +1808,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="22" spans="2:18" hidden="1">
+    <row r="22" spans="2:18">
       <c r="B22" t="s">
         <v>87</v>
       </c>
@@ -2026,7 +2144,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="31" spans="2:18" hidden="1">
+    <row r="31" spans="2:18">
       <c r="B31" t="s">
         <v>85</v>
       </c>
@@ -2065,10 +2183,11 @@
     <hyperlink ref="Q30" r:id="rId2" xr:uid="{BE22F3F0-2846-435C-B6CA-0BD8493B6880}"/>
     <hyperlink ref="Q29" r:id="rId3" xr:uid="{80A311A9-14ED-4AD4-8FFC-1270B33C2666}"/>
     <hyperlink ref="Q14" r:id="rId4" xr:uid="{5CE7C215-8E78-48EA-A2DF-1275BB4C83E4}"/>
+    <hyperlink ref="Q19" r:id="rId5" xr:uid="{D235CEED-9DC3-4E86-B456-9A68D7BB8D65}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
implemented media village and olympic village in popualtion files of Fast Track scenario
</commit_message>
<xml_diff>
--- a/original-input-data/mvv_gtfs_2037/Infrastructure_measures.xlsx
+++ b/original-input-data/mvv_gtfs_2037/Infrastructure_measures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DavidBerling\Masterarbeit Lokal\WP2\Matsim-example-project-TU-Kurs\original-input-data\mvv_gtfs_2037\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85952E1-3C3F-4B1C-832D-3032A38B1162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7412925D-FBA9-4B4A-89A2-D5446DBC4B48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6983" yWindow="-16297" windowWidth="28995" windowHeight="15675" xr2:uid="{C9EB77A7-838A-4CDA-9FC2-6F0F3DBDABA8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="194">
   <si>
     <t>Definition BAU and FT:
 - Im BAU 2040 werden nur Maßnahmen berücksichtigt, deren Umsetzung bis 2040 bereits unabhängig von einer Olympiabewerbung hinreichend gesichert oder sehr plausibel ist.
@@ -636,6 +636,36 @@
   </si>
   <si>
     <t>S20</t>
+  </si>
+  <si>
+    <t>population_2040.xml; home and work activities</t>
+  </si>
+  <si>
+    <t>Centroid proxy (WGS84): 48.142233, 11.657852; transform to EPSG:31468 before implementation</t>
+  </si>
+  <si>
+    <t>Target assumption: 3,500 residents and 1,167 jobs; 5% sample: relocate 175 persons by home location and 58 work activities</t>
+  </si>
+  <si>
+    <t>No new persons are generated. Total population, activity times, plan structure and existing mode choices remain unchanged</t>
+  </si>
+  <si>
+    <t>https://stadt.muenchen.de/dam/jcr:7b868e98-b9f0-4310-ac7c-32d1c4b526d6/PraesentationNordosten.pdf</t>
+  </si>
+  <si>
+    <t>The permanent post-Games land-use mix has not yet been officially defined. Therefore, the accommodation capacity of 3,500 media professionals is used as a proxy for permanent residents. The job target is derived from the MNO-wide ratio of one job per three residents. The centroid is a manually derived model proxy. Selected locations are relocated deterministically using a fixed random seed</t>
+  </si>
+  <si>
+    <t>Centroid proxy (WGS84): 48.153739, 11.658821; transform to EPSG:31468 before implementation</t>
+  </si>
+  <si>
+    <t>Target: 10,500 residents and 3,500 jobs; 5% sample: relocate 525 persons by home location and 175 work activities</t>
+  </si>
+  <si>
+    <t>No new persons are generated. Total population, activity times, plan structure and existing mode choices remain unchanged.</t>
+  </si>
+  <si>
+    <t>The centroid is a model proxy manually derived from the official planning map, not an officially defined site centre. The residential target follows the published estimate of approximately 4,000 dwellings and 10,500 residents. The job target is derived from the MNO-wide ratio of 10,000 jobs to 30,000 residents. Selected locations are relocated deterministically using a fixed random seed.</t>
   </si>
 </sst>
 </file>
@@ -798,19 +828,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{61883FC4-1D17-4081-8945-EF8683794370}" name="Tabelle4" displayName="Tabelle4" ref="A4:P31" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A4:P31" xr:uid="{61883FC4-1D17-4081-8945-EF8683794370}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="ja"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="7">
-      <filters>
-        <filter val="nein"/>
-        <filter val="teilweise"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A4:P31" xr:uid="{61883FC4-1D17-4081-8945-EF8683794370}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:K31">
     <sortCondition ref="C4:C31"/>
   </sortState>
@@ -1345,7 +1363,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="14.4" hidden="1" customHeight="1">
+    <row r="10" spans="1:18" ht="14.4" customHeight="1">
       <c r="B10" t="s">
         <v>38</v>
       </c>
@@ -1371,7 +1389,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="14.4" hidden="1" customHeight="1">
+    <row r="11" spans="1:18" ht="14.4" customHeight="1">
       <c r="B11" t="s">
         <v>41</v>
       </c>
@@ -1398,7 +1416,7 @@
       </c>
       <c r="L11" s="7"/>
     </row>
-    <row r="12" spans="1:18" ht="14.4" hidden="1" customHeight="1">
+    <row r="12" spans="1:18" ht="14.4" customHeight="1">
       <c r="B12" t="s">
         <v>44</v>
       </c>
@@ -1573,7 +1591,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="16" spans="1:18" hidden="1">
+    <row r="16" spans="1:18">
       <c r="B16" t="s">
         <v>79</v>
       </c>
@@ -1770,8 +1788,23 @@
       <c r="L20" t="s">
         <v>136</v>
       </c>
-      <c r="M20" t="s">
-        <v>134</v>
+      <c r="M20" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="N20" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="O20" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="P20" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>188</v>
+      </c>
+      <c r="R20" s="13" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="21" spans="2:18">
@@ -1804,8 +1837,23 @@
       <c r="L21" t="s">
         <v>136</v>
       </c>
-      <c r="M21" t="s">
-        <v>134</v>
+      <c r="M21" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="N21" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="O21" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="P21" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>188</v>
+      </c>
+      <c r="R21" s="13" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="2:18">
@@ -1837,7 +1885,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="23" spans="2:18" hidden="1">
+    <row r="23" spans="2:18">
       <c r="B23" t="s">
         <v>71</v>
       </c>
@@ -1869,7 +1917,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="24" spans="2:18" hidden="1">
+    <row r="24" spans="2:18">
       <c r="B24" t="s">
         <v>75</v>
       </c>
@@ -1901,7 +1949,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="25" spans="2:18" hidden="1">
+    <row r="25" spans="2:18">
       <c r="B25" t="s">
         <v>77</v>
       </c>
@@ -1933,7 +1981,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="26" spans="2:18" hidden="1">
+    <row r="26" spans="2:18">
       <c r="B26" t="s">
         <v>18</v>
       </c>
@@ -1968,7 +2016,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="27" spans="2:18" hidden="1">
+    <row r="27" spans="2:18">
       <c r="B27" t="s">
         <v>24</v>
       </c>
@@ -2003,7 +2051,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="28" spans="2:18" hidden="1">
+    <row r="28" spans="2:18">
       <c r="B28" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
pedestrian zones for fast track implemented
</commit_message>
<xml_diff>
--- a/original-input-data/mvv_gtfs_2037/Infrastructure_measures.xlsx
+++ b/original-input-data/mvv_gtfs_2037/Infrastructure_measures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DavidBerling\Masterarbeit Lokal\WP2\Matsim-example-project-TU-Kurs\original-input-data\mvv_gtfs_2037\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7412925D-FBA9-4B4A-89A2-D5446DBC4B48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188707BC-C75F-4078-8D7E-B7CC85ACC55B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6983" yWindow="-16297" windowWidth="28995" windowHeight="15675" xr2:uid="{C9EB77A7-838A-4CDA-9FC2-6F0F3DBDABA8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="195">
   <si>
     <t>Definition BAU and FT:
 - Im BAU 2040 werden nur Maßnahmen berücksichtigt, deren Umsetzung bis 2040 bereits unabhängig von einer Olympiabewerbung hinreichend gesichert oder sehr plausibel ist.
@@ -666,6 +666,9 @@
   </si>
   <si>
     <t>The centroid is a model proxy manually derived from the official planning map, not an officially defined site centre. The residential target follows the published estimate of approximately 4,000 dwellings and 10,500 residents. The job target is derived from the MNO-wide ratio of 10,000 jobs to 30,000 residents. Selected locations are relocated deterministically using a fixed random seed.</t>
+  </si>
+  <si>
+    <t>nicht berücksichtigen</t>
   </si>
 </sst>
 </file>
@@ -1876,7 +1879,7 @@
         <v>33</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>107</v>
+        <v>194</v>
       </c>
       <c r="J22" s="10" t="s">
         <v>117</v>
@@ -1884,6 +1887,7 @@
       <c r="L22" t="s">
         <v>134</v>
       </c>
+      <c r="R22" s="13"/>
     </row>
     <row r="23" spans="2:18">
       <c r="B23" t="s">

</xml_diff>